<commit_message>
physician package: human-readable rule statements
</commit_message>
<xml_diff>
--- a/eval/human/Hemoglyph_physician_review_package_v1.xlsx
+++ b/eval/human/Hemoglyph_physician_review_package_v1.xlsx
@@ -19661,12 +19661,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{"all": [{"feature_id": "serum_protein_electrophoresis_m_spike", "operator": "&gt;=", "value": 3.0, "unit": "g/dL", "weight": 3.0}, {"any": [{"feature_id": "corrected_calcium_for_serum_albumin", "operator": "&gt;", "value": 11.0, "unit": "mg/dL", "weight": 3.0}, {"feature_id": "calcium_total", "operator": "&gt;", "value": 11.0, "unit": "mg/dL", "weight": 3.0}, {"feature_id": "creatinine", "operator": "&gt;", "value": 2.0, "unit": "mg/dL", "weight": 3.0}, {"feature_id": "hemoglobin", "operator": "&lt;", "value": 10.0, "unit": "g/dL", "weight": 3.0}]}]}</t>
+          <t>(serum_protein_electrophoresis_m_spike &gt;= 3.0 g/dL) AND ((corrected_calcium_for_serum_albumin &gt; 11.0 mg/dL) OR (calcium_total &gt; 11.0 mg/dL) OR (creatinine &gt; 2.0 mg/dL) OR (hemoglobin &lt; 10.0 g/dL))</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>{"age_groups": ["adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>adolescent, adult, older_adult; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -19710,12 +19710,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{"all": [{"feature_id": "indirect_bilirubin", "operator": "&gt;", "value": 1.0, "unit": "mg/dL", "weight": 3.0}, {"feature_id": "lactate_dehydrogenase", "operator": "&gt;", "value": 250.0, "unit": "U/L", "weight": 3.0}, {"feature_id": "serum_haptoglobin", "operator": "&lt;", "value": 30.0, "unit": "mg/dL", "weight": 3.0}]}</t>
+          <t>(indirect_bilirubin &gt; 1.0 mg/dL) AND (lactate_dehydrogenase &gt; 250.0 U/L) AND (serum_haptoglobin &lt; 30.0 mg/dL)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -19759,12 +19759,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{"any": [{"feature_id": "vitamin_b12", "operator": "&lt;", "value": 148, "unit": "pg/mL", "weight": 3.0}, {"all": [{"feature_id": "vitamin_b12", "operator": "&lt;", "value": 200, "unit": "pg/mL", "weight": 3.0}, {"feature_id": "methylmalonic_acid", "operator": "&gt;", "value": 271, "unit": "ng/mL", "weight": 3.0}]}]}</t>
+          <t>(vitamin_b12 &lt; 148 pg/mL) OR ((vitamin_b12 &lt; 200 pg/mL) AND (methylmalonic_acid &gt; 271 ng/mL))</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -19808,12 +19808,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{"all": [{"feature_id": "coombs_direct_antiglobulin_test", "operator": "==", "value": 1, "unit": "1", "weight": 3.0}, {"feature_id": "haptoglobin_serum_quantitative", "operator": "&lt;", "value": 25, "unit": "mg/dL", "weight": 3.0}, {"feature_id": "hemoglobin", "operator": "&lt;", "value": 10.67, "unit": "g/dL", "weight": 3.0}]}</t>
+          <t>(coombs_direct_antiglobulin_test == 1 1) AND (haptoglobin_serum_quantitative &lt; 25 mg/dL) AND (hemoglobin &lt; 10.67 g/dL)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "female", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: female; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -19857,12 +19857,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{"all": [{"feature_id": "platelets", "operator": "&lt;", "value": 30, "unit": "10*9/L", "weight": 3.0}, {"feature_id": "lactate_dehydrogenase", "operator": "&gt;", "value": 500, "unit": "U/L", "weight": 3.0}, {"feature_id": "haptoglobin_serum_quantitative", "operator": "&lt;", "value": 25, "unit": "mg/dL", "weight": 3.0}, {"feature_id": "creatinine", "operator": "&lt;", "value": 2.0, "unit": "mg/dL", "weight": 3.0}]}</t>
+          <t>(platelets &lt; 30 10*9/L) AND (lactate_dehydrogenase &gt; 500 U/L) AND (haptoglobin_serum_quantitative &lt; 25 mg/dL) AND (creatinine &lt; 2.0 mg/dL)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -19906,12 +19906,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{"all": [{"any": [{"feature_id": "lactate_dehydrogenase", "operator": "&gt;", "value": 250, "unit": "U/L", "weight": 3.0}, {"feature_id": "indirect_bilirubin", "operator": "&gt;", "value": 1.0, "unit": "mg/dL", "weight": 3.0}]}, {"feature_id": "haptoglobin_serum_quantitative", "operator": "&lt;", "value": 25, "unit": "mg/dL", "weight": 3.0}, {"any": [{"feature_id": "reticulocytes", "operator": "&gt;", "value": 2.5, "unit": "%", "weight": 3.0}, {"feature_id": "hemoglobin", "operator": "&lt;", "value": 12.0, "unit": "g/dL", "weight": 3.0}]}]}</t>
+          <t>((lactate_dehydrogenase &gt; 250 U/L) OR (indirect_bilirubin &gt; 1.0 mg/dL)) AND (haptoglobin_serum_quantitative &lt; 25 mg/dL) AND ((reticulocytes &gt; 2.5 %) OR (hemoglobin &lt; 12.0 g/dL))</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -19955,12 +19955,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{"all": [{"any": [{"feature_id": "hemoglobin", "operator": "&gt;", "value": 16.5, "unit": "g/dL", "weight": 3.0}, {"feature_id": "hematocrit", "operator": "&gt;", "value": 49, "unit": "%", "weight": 3.0}]}, {"feature_id": "jak2_v617f_mutation", "operator": "==", "value": 1, "unit": "1", "weight": 3.0}]}</t>
+          <t>((hemoglobin &gt; 16.5 g/dL) OR (hematocrit &gt; 49 %)) AND (jak2_v617f_mutation == 1 1)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -20004,12 +20004,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{"all": [{"any": [{"feature_id": "lactate_dehydrogenase", "operator": "&gt;", "value": 250, "unit": "U/L", "weight": 3.0}, {"feature_id": "indirect_bilirubin", "operator": "&gt;", "value": 1.0, "unit": "mg/dL", "weight": 3.0}]}, {"feature_id": "haptoglobin_serum_quantitative", "operator": "&lt;", "value": 25, "unit": "mg/dL", "weight": 3.0}, {"any": [{"feature_id": "reticulocytes", "operator": "&gt;", "value": 2.5, "unit": "%", "weight": 3.0}, {"feature_id": "hemoglobin", "operator": "&lt;", "value": 10.67, "unit": "g/dL", "weight": 3.0}]}]}</t>
+          <t>((lactate_dehydrogenase &gt; 250 U/L) OR (indirect_bilirubin &gt; 1.0 mg/dL)) AND (haptoglobin_serum_quantitative &lt; 25 mg/dL) AND ((reticulocytes &gt; 2.5 %) OR (hemoglobin &lt; 10.67 g/dL))</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "female", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: female; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -20053,12 +20053,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin_s", "operator": "&gt;", "value": 50, "unit": "%", "weight": 3.0}</t>
+          <t>hemoglobin_s &gt; 50 %</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -20102,12 +20102,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{"all": [{"feature_id": "ferritin", "operator": "&lt;", "value": 100, "unit": "ng/mL", "weight": 3.0}, {"feature_id": "transferrin_saturation", "operator": "&lt;", "value": 20, "unit": "%", "weight": 3.0}, {"feature_id": "c_reactive_protein", "operator": "&gt;", "value": 5, "unit": "mg/L", "weight": 3.0}, {"feature_id": "hemoglobin", "operator": "&lt;", "value": 12.0, "unit": "g/dL", "weight": 3.0}]}</t>
+          <t>(ferritin &lt; 100 ng/mL) AND (transferrin_saturation &lt; 20 %) AND (c_reactive_protein &gt; 5 mg/L) AND (hemoglobin &lt; 12.0 g/dL)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -20151,12 +20151,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>{"any": [{"feature_id": "free_kappa_to_lambda_ratio", "operator": "&gt;=", "value": 100.0, "unit": "1", "weight": 3.0}, {"feature_id": "free_kappa_to_lambda_ratio", "operator": "&lt;=", "value": 0.01, "unit": "1", "weight": 3.0}, {"feature_id": "monoclonal_protein_quantitation", "operator": "&gt;=", "value": 3000.0, "unit": "mg/dL", "weight": 3.0}]}</t>
+          <t>(free_kappa_to_lambda_ratio &gt;= 100.0 1) OR (free_kappa_to_lambda_ratio &lt;= 0.01 1) OR (monoclonal_protein_quantitation &gt;= 3000.0 mg/dL)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -20200,12 +20200,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>{"feature_id": "platelets", "operator": "&gt;=", "value": 450, "unit": "10*9/L", "weight": 3.0}</t>
+          <t>platelets &gt;= 450 10*9/L</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -20249,12 +20249,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -20298,12 +20298,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -20347,12 +20347,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -20396,12 +20396,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -20445,12 +20445,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -20494,12 +20494,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{"all": [{"feature_id": "hemoglobin", "operator": "&lt;", "value": 10.67, "unit": "g/dL", "weight": 3.0}, {"feature_id": "ferritin", "operator": "&lt;", "value": 15.0, "unit": "ng/mL", "weight": 3.0}]}</t>
+          <t>(hemoglobin &lt; 10.67 g/dL) AND (ferritin &lt; 15.0 ng/mL)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "female", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: female; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -20543,12 +20543,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>{"feature_id": "total_bilirubin", "operator": "&gt;=", "value": 2.5, "unit": "mg/dL", "weight": 6.0}</t>
+          <t>total_bilirubin &gt;= 2.5 mg/dL</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -20592,12 +20592,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 9.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 9.0 g/dL</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -20641,12 +20641,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 10.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 10.0 g/dL</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -20690,12 +20690,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -20739,12 +20739,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -20788,12 +20788,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 7.0, "unit": "g/dL", "weight": 5.0}</t>
+          <t>hemoglobin &lt; 7.0 g/dL</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -20837,12 +20837,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>{"all": [{"feature_id": "hemoglobin", "operator": "&lt;", "value": 10.67, "unit": "g/dL", "weight": 2.0}, {"feature_id": "mean_corpuscular_volume", "operator": "&gt;", "value": 100.0, "unit": "fL", "weight": 2.0}, {"feature_id": "vitamin_b12", "operator": "&lt;", "value": 200.0, "unit": "pg/mL", "weight": 2.0}]}</t>
+          <t>(hemoglobin &lt; 10.67 g/dL) AND (mean_corpuscular_volume &gt; 100.0 fL) AND (vitamin_b12 &lt; 200.0 pg/mL)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child", "adolescent", "adult", "older_adult"], "sex": "female", "pregnancy": "context_dependent"}</t>
+          <t>child, adolescent, adult, older_adult; sex: female; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -20886,12 +20886,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 13.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 13.0 g/dL</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>{"age_groups": ["neonate", "infant", "child", "adolescent", "adult", "older_adult"], "sex": "male", "pregnancy": "context_dependent"}</t>
+          <t>all ages; sex: male; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -20935,12 +20935,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>{"feature_id": "hemoglobin", "operator": "&lt;", "value": 10.0, "unit": "g/dL", "weight": 3.0}</t>
+          <t>hemoglobin &lt; 10.0 g/dL</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>{"age_groups": ["child"], "sex": "all", "pregnancy": "context_dependent"}</t>
+          <t>child; sex: all; pregnancy: context_dependent</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">

</xml_diff>